<commit_message>
Primeiros testes de programação orientada a objeto
</commit_message>
<xml_diff>
--- a/Necessario/Financeiro_novo.xlsx
+++ b/Necessario/Financeiro_novo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -988,6 +988,66 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Débito</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Lanche</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Débito</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>